<commit_message>
[feature] added nonstandard properties to expansion joint entity
</commit_message>
<xml_diff>
--- a/IFC_Converter.xlsx
+++ b/IFC_Converter.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\glebf\source\repos\IFC_Converter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{694EE7E2-6A1D-4EAB-8E4E-13735FC313F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D16E413F-7C87-40C6-8EF3-D7A756E310F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WindowTranslations" sheetId="1" r:id="rId1"/>
     <sheet name="Properties" sheetId="2" r:id="rId2"/>
+    <sheet name="Entities" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="267">
   <si>
     <t>DirectoryDoesNotExists_Error</t>
   </si>
@@ -602,6 +603,231 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>Name (EN)</t>
+  </si>
+  <si>
+    <t>Name (RU)</t>
+  </si>
+  <si>
+    <t>Заглушка</t>
+  </si>
+  <si>
+    <t>Арматура</t>
+  </si>
+  <si>
+    <t>Фланцевое соединение</t>
+  </si>
+  <si>
+    <t>Одиночный фланец</t>
+  </si>
+  <si>
+    <t>Соединение</t>
+  </si>
+  <si>
+    <t>Участок трубы</t>
+  </si>
+  <si>
+    <t>Жесткая вставка</t>
+  </si>
+  <si>
+    <t>Цилиндрическая обечайка</t>
+  </si>
+  <si>
+    <t>Балка</t>
+  </si>
+  <si>
+    <t>Гибкая вставка</t>
+  </si>
+  <si>
+    <t>Конус</t>
+  </si>
+  <si>
+    <t>Участки</t>
+  </si>
+  <si>
+    <t>Оборудование</t>
+  </si>
+  <si>
+    <t>Штуцер WRC 107/537/197</t>
+  </si>
+  <si>
+    <t>Штуцер резервуара API 650</t>
+  </si>
+  <si>
+    <t>Насос гост 32601 / API 650 / ISO 13709</t>
+  </si>
+  <si>
+    <t>Насос гост p. 54806 / ISO 9905</t>
+  </si>
+  <si>
+    <t>Насос гост p. 54805 / ISO 5199</t>
+  </si>
+  <si>
+    <t>Инлайн насос</t>
+  </si>
+  <si>
+    <t>Другой насос</t>
+  </si>
+  <si>
+    <t>Турбина</t>
+  </si>
+  <si>
+    <t>Компрессор</t>
+  </si>
+  <si>
+    <t>Аппарат воздушного охлаждения</t>
+  </si>
+  <si>
+    <t>Отвод</t>
+  </si>
+  <si>
+    <t>Кругоизогнутый</t>
+  </si>
+  <si>
+    <t>Гнутый</t>
+  </si>
+  <si>
+    <t>Секторный</t>
+  </si>
+  <si>
+    <t>Штампосварной</t>
+  </si>
+  <si>
+    <t>Гнутый большого радиуса</t>
+  </si>
+  <si>
+    <t>Упруго-изогнутый участок</t>
+  </si>
+  <si>
+    <t>Косой стык</t>
+  </si>
+  <si>
+    <t>Подпятник</t>
+  </si>
+  <si>
+    <t>Нестандартный отвод</t>
+  </si>
+  <si>
+    <t>Печь</t>
+  </si>
+  <si>
+    <t>Тройник</t>
+  </si>
+  <si>
+    <t>Сварной (кованный)</t>
+  </si>
+  <si>
+    <t>Врезка</t>
+  </si>
+  <si>
+    <t>Тройник с вытянутой горловинной</t>
+  </si>
+  <si>
+    <t>Велдолет (с усиленным штуцером)</t>
+  </si>
+  <si>
+    <t>Свеполет (с вварным кольцом)</t>
+  </si>
+  <si>
+    <t>Пластиковый тройник</t>
+  </si>
+  <si>
+    <t>Стойка</t>
+  </si>
+  <si>
+    <t>Нестандартный тройник</t>
+  </si>
+  <si>
+    <t>Переход</t>
+  </si>
+  <si>
+    <t>Концентрический</t>
+  </si>
+  <si>
+    <t>Эксцентрический</t>
+  </si>
+  <si>
+    <t>Крепление</t>
+  </si>
+  <si>
+    <t>Неподвижная опора (метвая)</t>
+  </si>
+  <si>
+    <t>Шарнирно-неподвижная опора</t>
+  </si>
+  <si>
+    <t>Скользящая опора</t>
+  </si>
+  <si>
+    <t>Пружинная опора</t>
+  </si>
+  <si>
+    <t>Пружинная подвеска</t>
+  </si>
+  <si>
+    <t>Направляющая опора двусторонняя</t>
+  </si>
+  <si>
+    <t>Направляющая опора односторонняя</t>
+  </si>
+  <si>
+    <t>Жесткая подвеска / стойка</t>
+  </si>
+  <si>
+    <t>Опора постоянного усилия</t>
+  </si>
+  <si>
+    <t>Подвеска постоянного усилия</t>
+  </si>
+  <si>
+    <t>Нестандартное крепление</t>
+  </si>
+  <si>
+    <t>Демпфер</t>
+  </si>
+  <si>
+    <t>Амортизатор</t>
+  </si>
+  <si>
+    <t>Компенсатор</t>
+  </si>
+  <si>
+    <t>Осевой стартовый</t>
+  </si>
+  <si>
+    <t>Осевой сильфонный</t>
+  </si>
+  <si>
+    <t>Осевой сальниковый</t>
+  </si>
+  <si>
+    <t>Осевой линзовый</t>
+  </si>
+  <si>
+    <t>Осевая муфта</t>
+  </si>
+  <si>
+    <t>Универсальный</t>
+  </si>
+  <si>
+    <t>Угловой карданный</t>
+  </si>
+  <si>
+    <t>Угловой крутильный</t>
+  </si>
+  <si>
+    <t>Шаровой</t>
+  </si>
+  <si>
+    <t>Сдвиговый</t>
+  </si>
+  <si>
+    <t>Нестандартный</t>
+  </si>
+  <si>
+    <t>Масса</t>
   </si>
 </sst>
 </file>
@@ -634,12 +860,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -654,30 +892,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="5">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <charset val="204"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <charset val="204"/>
-      </font>
-    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -697,6 +925,18 @@
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <charset val="204"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <charset val="204"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -744,11 +984,11 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{153D1ECA-3A1A-42AD-B2C6-A259002DDB4B}" name="Таблица2" displayName="Таблица2" ref="B1:E112" totalsRowShown="0" headerRowDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{153D1ECA-3A1A-42AD-B2C6-A259002DDB4B}" name="Таблица2" displayName="Таблица2" ref="B1:E112" totalsRowShown="0" headerRowDxfId="3">
   <autoFilter ref="B1:E112" xr:uid="{153D1ECA-3A1A-42AD-B2C6-A259002DDB4B}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{307D036C-F783-44DB-B2C5-47A9E148305D}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{3F5F3928-FA53-45DF-970F-BBD070757265}" name="Name" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{3F5F3928-FA53-45DF-970F-BBD070757265}" name="Name" dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{9A1BE7E0-560F-44DA-83FE-97472CA273C7}" name="StartUnits"/>
     <tableColumn id="4" xr3:uid="{72005284-6376-412A-8F16-762E37F0866A}" name="SIUnits"/>
   </tableColumns>
@@ -2842,8 +3082,8 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:B112">
-    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -2851,4 +3091,397 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5C43E16-497E-42EA-84A4-608642D8B623}">
+  <dimension ref="B2:C76"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C3" s="4" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C4" s="4" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C5" s="4" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C7" s="4" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C8" s="2" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C9" s="4" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C10" s="4" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C11" s="4" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C12" s="5" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C13" s="4" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C14" s="4" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C15" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C16" s="4" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="17" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C17" s="4" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="18" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C18" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="19" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C19" s="4" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="20" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C20" s="4" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="21" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C21" s="4" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="22" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C22" s="4" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="23" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C23" s="4" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="24" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C24" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="25" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C25" s="4" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="26" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C26" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="27" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C27" s="2" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="28" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C28" s="4" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="29" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C29" s="4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="30" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C30" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="31" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C31" s="4" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="32" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C32" s="4" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C33" s="4" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C34" s="4" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="35" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C35" s="4" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="36" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C36" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="37" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C37" s="2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="38" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C38" s="4" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="39" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C39" s="4" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="40" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C40" s="4" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="41" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C41" s="4" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="42" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C42" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="43" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C43" s="4" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="44" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C44" s="4" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="45" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C45" s="4" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="46" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C46" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="47" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C47" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="48" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C48" s="4" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="49" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C49" s="4" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="50" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C50" s="2" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="51" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C51" s="4" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="52" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C52" s="4" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="53" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C53" s="4" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="54" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C54" s="4" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="55" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C55" s="4" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="56" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C56" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="57" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C57" s="4" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="58" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C58" s="4" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="59" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C59" s="4" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="60" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C60" s="4" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="61" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C61" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="62" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C62" s="4" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="63" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C63" s="4" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="64" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C64" s="2" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="65" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C65" s="4" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="66" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C66" s="4" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="67" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C67" s="4" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="68" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C68" s="4" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="69" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C69" s="4" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="70" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C70" s="4" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="71" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C71" s="4" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="72" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C72" s="4" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="73" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C73" s="4" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="74" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C74" s="4" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="75" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C75" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="76" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C76" t="s">
+        <v>266</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
[feature] added nonstandard tee entity convert
</commit_message>
<xml_diff>
--- a/IFC_Converter.xlsx
+++ b/IFC_Converter.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\glebf\source\repos\IFC_Converter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D16E413F-7C87-40C6-8EF3-D7A756E310F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE904D08-7BA3-47D6-97B2-C5232E329095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -908,6 +908,18 @@
   <dxfs count="5">
     <dxf>
       <font>
+        <b val="0"/>
+        <charset val="204"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <charset val="204"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -925,18 +937,6 @@
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <charset val="204"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <charset val="204"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -984,11 +984,11 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{153D1ECA-3A1A-42AD-B2C6-A259002DDB4B}" name="Таблица2" displayName="Таблица2" ref="B1:E112" totalsRowShown="0" headerRowDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{153D1ECA-3A1A-42AD-B2C6-A259002DDB4B}" name="Таблица2" displayName="Таблица2" ref="B1:E112" totalsRowShown="0" headerRowDxfId="1">
   <autoFilter ref="B1:E112" xr:uid="{153D1ECA-3A1A-42AD-B2C6-A259002DDB4B}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{307D036C-F783-44DB-B2C5-47A9E148305D}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{3F5F3928-FA53-45DF-970F-BBD070757265}" name="Name" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{3F5F3928-FA53-45DF-970F-BBD070757265}" name="Name" dataDxfId="0"/>
     <tableColumn id="3" xr3:uid="{9A1BE7E0-560F-44DA-83FE-97472CA273C7}" name="StartUnits"/>
     <tableColumn id="4" xr3:uid="{72005284-6376-412A-8F16-762E37F0866A}" name="SIUnits"/>
   </tableColumns>
@@ -3082,8 +3082,8 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:B112">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -3326,7 +3326,7 @@
       </c>
     </row>
     <row r="46" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C46" t="s">
+      <c r="C46" s="4" t="s">
         <v>236</v>
       </c>
     </row>
@@ -3471,7 +3471,7 @@
       </c>
     </row>
     <row r="75" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C75" t="s">
+      <c r="C75" s="4" t="s">
         <v>265</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[fix] fixed angular expansion joint
</commit_message>
<xml_diff>
--- a/IFC_Converter.xlsx
+++ b/IFC_Converter.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\glebf\source\repos\IFC_Converter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE904D08-7BA3-47D6-97B2-C5232E329095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5758A872-3977-4966-A1FB-C803A4DE5469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="273">
   <si>
     <t>DirectoryDoesNotExists_Error</t>
   </si>
@@ -828,6 +828,24 @@
   </si>
   <si>
     <t>Масса</t>
+  </si>
+  <si>
+    <t>Cap</t>
+  </si>
+  <si>
+    <t>Armature</t>
+  </si>
+  <si>
+    <t>Rigid Element</t>
+  </si>
+  <si>
+    <t>Pipe Segment</t>
+  </si>
+  <si>
+    <t>Cylindrical Shell</t>
+  </si>
+  <si>
+    <t>Cone Element</t>
   </si>
 </sst>
 </file>
@@ -3098,8 +3116,8 @@
   <dimension ref="B2:C76"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:3" x14ac:dyDescent="0.25">
@@ -3111,11 +3129,17 @@
       </c>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>267</v>
+      </c>
       <c r="C3" s="4" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>268</v>
+      </c>
       <c r="C4" s="4" t="s">
         <v>195</v>
       </c>
@@ -3126,7 +3150,7 @@
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C6" t="s">
+      <c r="C6" s="4" t="s">
         <v>197</v>
       </c>
     </row>
@@ -3141,16 +3165,25 @@
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>270</v>
+      </c>
       <c r="C9" s="4" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>269</v>
+      </c>
       <c r="C10" s="4" t="s">
         <v>200</v>
       </c>
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>271</v>
+      </c>
       <c r="C11" s="4" t="s">
         <v>201</v>
       </c>
@@ -3166,6 +3199,9 @@
       </c>
     </row>
     <row r="14" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>272</v>
+      </c>
       <c r="C14" s="4" t="s">
         <v>204</v>
       </c>
@@ -3226,7 +3262,7 @@
       </c>
     </row>
     <row r="26" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C26" t="s">
+      <c r="C26" s="4" t="s">
         <v>227</v>
       </c>
     </row>
@@ -3276,7 +3312,7 @@
       </c>
     </row>
     <row r="36" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C36" t="s">
+      <c r="C36" s="4" t="s">
         <v>226</v>
       </c>
     </row>
@@ -3401,7 +3437,7 @@
       </c>
     </row>
     <row r="61" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C61" t="s">
+      <c r="C61" s="4" t="s">
         <v>251</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[feature] added fittings convert
</commit_message>
<xml_diff>
--- a/IFC_Converter.xlsx
+++ b/IFC_Converter.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\glebf\source\repos\IFC_Converter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F49A075-88B4-4A5D-82D0-448BF976EA50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BC572C6-EE5E-48E4-B508-187C86C63E12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="273">
   <si>
     <t>DirectoryDoesNotExists_Error</t>
   </si>
@@ -3113,22 +3113,25 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5C43E16-497E-42EA-84A4-608642D8B623}">
-  <dimension ref="B2:C76"/>
+  <dimension ref="B2:D76"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="36.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>192</v>
       </c>
       <c r="C2" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>267</v>
       </c>
@@ -3136,7 +3139,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>268</v>
       </c>
@@ -3144,74 +3147,89 @@
         <v>195</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C5" s="4" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C6" s="4" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C7" s="4" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C8" s="2" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>270</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>269</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>271</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C12" s="5" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C13" s="4" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D13">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>272</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D14">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C15" s="2" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C16" s="4" t="s">
         <v>207</v>
       </c>
@@ -3376,82 +3394,106 @@
         <v>238</v>
       </c>
     </row>
-    <row r="49" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C49" s="4" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="50" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C50" s="2" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="51" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C51" s="4" t="s">
         <v>241</v>
       </c>
-    </row>
-    <row r="52" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="D51">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="52" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C52" s="4" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="53" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C53" s="4" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="54" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="D53">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="54" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C54" s="4" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="55" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="D54">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="55" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C55" s="4" t="s">
         <v>245</v>
       </c>
-    </row>
-    <row r="56" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="D55">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="56" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C56" s="4" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="57" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="D56">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="57" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C57" s="4" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="58" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="D57">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="58" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C58" s="4" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="59" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C59" s="4" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="60" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C60" s="4" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="61" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="D60">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="61" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C61" s="4" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="62" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C62" s="4" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="63" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="D62">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="63" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C63" s="4" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="64" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C64" s="2" t="s">
         <v>254</v>
       </c>

</xml_diff>

<commit_message>
[feature] added data array init from StartAutoServer [fix] fixed CTAPT version in IFCProject
</commit_message>
<xml_diff>
--- a/IFC_Converter.xlsx
+++ b/IFC_Converter.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\glebf\source\repos\IFC_Converter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BC572C6-EE5E-48E4-B508-187C86C63E12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75AAF242-975F-4B05-A2EF-6E2CD046ACCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WindowTranslations" sheetId="1" r:id="rId1"/>
@@ -22,12 +22,15 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="290">
   <si>
     <t>DirectoryDoesNotExists_Error</t>
   </si>
@@ -846,6 +849,57 @@
   </si>
   <si>
     <t>Cone Element</t>
+  </si>
+  <si>
+    <t>ImportWindowForm_selectInputFilePathButton_Text</t>
+  </si>
+  <si>
+    <t>ImportWindowForm_Text</t>
+  </si>
+  <si>
+    <t>ImportWindowForm_ImportButton_Text</t>
+  </si>
+  <si>
+    <t>ImportWindowForm_InputFilePath_Label_Text</t>
+  </si>
+  <si>
+    <t>ImportWindowForm_ImportType_Label_Text</t>
+  </si>
+  <si>
+    <t>ImportWindowForm_ImportType_Error</t>
+  </si>
+  <si>
+    <t>ImportWindowForm_InputFilePath_Empty_Error</t>
+  </si>
+  <si>
+    <t>ImportWindowForm_ImportType_Aveva</t>
+  </si>
+  <si>
+    <t>Import</t>
+  </si>
+  <si>
+    <t>Импорт</t>
+  </si>
+  <si>
+    <t>Import profile</t>
+  </si>
+  <si>
+    <t>Enter a full path of IFC file to be imported</t>
+  </si>
+  <si>
+    <t>Укажите полный путь для импорта .ifc файла</t>
+  </si>
+  <si>
+    <t>Профиль импорта</t>
+  </si>
+  <si>
+    <t>Unknown import type</t>
+  </si>
+  <si>
+    <t>Неизвестный тип импорта</t>
+  </si>
+  <si>
+    <t>AVEVA</t>
   </si>
 </sst>
 </file>
@@ -910,7 +964,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -919,21 +973,52 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="8">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
-        <b val="0"/>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
         <charset val="204"/>
+        <scheme val="minor"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <charset val="204"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike/>
       </font>
     </dxf>
     <dxf>
@@ -958,21 +1043,14 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <charset val="204"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
         <charset val="204"/>
-        <scheme val="minor"/>
       </font>
     </dxf>
   </dxfs>
@@ -989,10 +1067,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3BE89974-193A-476A-B6D8-7855AC80A494}" name="Таблица1" displayName="Таблица1" ref="B1:E16" totalsRowShown="0">
-  <autoFilter ref="B1:E16" xr:uid="{3BE89974-193A-476A-B6D8-7855AC80A494}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3BE89974-193A-476A-B6D8-7855AC80A494}" name="Таблица1" displayName="Таблица1" ref="B1:E24" totalsRowShown="0">
+  <autoFilter ref="B1:E24" xr:uid="{3BE89974-193A-476A-B6D8-7855AC80A494}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{C53C5A7C-146B-44E6-94BA-B3CFC314CDA6}" name="ID" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{C53C5A7C-146B-44E6-94BA-B3CFC314CDA6}" name="ID" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{84A50B8C-BC4D-4680-9FFB-917ADF7F1A81}" name="English"/>
     <tableColumn id="3" xr3:uid="{7F2D5197-5510-45D3-A794-EA073700EC3F}" name="Russian"/>
     <tableColumn id="4" xr3:uid="{1DAAB3F8-FA67-43BC-A815-25370BF58753}" name="Chinese"/>
@@ -1002,11 +1080,11 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{153D1ECA-3A1A-42AD-B2C6-A259002DDB4B}" name="Таблица2" displayName="Таблица2" ref="B1:E112" totalsRowShown="0" headerRowDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{153D1ECA-3A1A-42AD-B2C6-A259002DDB4B}" name="Таблица2" displayName="Таблица2" ref="B1:E112" totalsRowShown="0" headerRowDxfId="7">
   <autoFilter ref="B1:E112" xr:uid="{153D1ECA-3A1A-42AD-B2C6-A259002DDB4B}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{307D036C-F783-44DB-B2C5-47A9E148305D}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{3F5F3928-FA53-45DF-970F-BBD070757265}" name="Name" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{3F5F3928-FA53-45DF-970F-BBD070757265}" name="Name" dataDxfId="6"/>
     <tableColumn id="3" xr3:uid="{9A1BE7E0-560F-44DA-83FE-97472CA273C7}" name="StartUnits"/>
     <tableColumn id="4" xr3:uid="{72005284-6376-412A-8F16-762E37F0866A}" name="SIUnits"/>
   </tableColumns>
@@ -1277,7 +1355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:E16"/>
+  <dimension ref="B1:E27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="51" bestFit="1" customWidth="1"/>
@@ -1484,33 +1562,143 @@
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="C15" t="s">
+        <v>28</v>
+      </c>
+      <c r="D15" t="s">
+        <v>43</v>
+      </c>
+      <c r="E15" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B16" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="C16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D16" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B17" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="C17" t="s">
+        <v>281</v>
+      </c>
+      <c r="D17" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B18" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="C18" t="s">
+        <v>284</v>
+      </c>
+      <c r="D18" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B19" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="C19" t="s">
+        <v>283</v>
+      </c>
+      <c r="D19" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B20" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="C20" t="s">
+        <v>287</v>
+      </c>
+      <c r="D20" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B21" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="C21" t="s">
+        <v>25</v>
+      </c>
+      <c r="D21" t="s">
+        <v>40</v>
+      </c>
+      <c r="E21" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B22" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="C22" t="s">
+        <v>289</v>
+      </c>
+      <c r="D22" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B23" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C23" t="s">
         <v>32</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D23" t="s">
         <v>47</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E23" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B16" s="2" t="s">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B24" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C24" t="s">
         <v>33</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D24" t="s">
         <v>48</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E24" t="s">
         <v>62</v>
       </c>
     </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B25" s="2"/>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B26" s="2"/>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B27" s="2"/>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="B2:B24">
+    <cfRule type="duplicateValues" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B1:B1048576">
+    <cfRule type="duplicateValues" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <tableParts count="1">
@@ -3100,8 +3288,8 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:B112">
-    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>

</xml_diff>